<commit_message>
Evento #2 registrado en reporte_2026-06-23.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-23.xlsx
+++ b/datos/excel/reporte_2026-06-23.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,51 @@
         <v>11750</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>09:56:37</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>335.94</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-18.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>648.4 Hz | 1023.4 Hz | 1375.0 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2533</v>
+      </c>
+      <c r="J3" t="n">
+        <v>62</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #1 registrado en reporte_2026-06-23.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-23.xlsx
+++ b/datos/excel/reporte_2026-06-23.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,51 @@
         <v>62</v>
       </c>
       <c r="K3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>09:57:36</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>328.12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-17.85</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>648.4 Hz | 968.8 Hz | 1281.2 Hz</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>2540</v>
+      </c>
+      <c r="J4" t="n">
+        <v>11955</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>